<commit_message>
religion added adn subjects final with dynamic year
</commit_message>
<xml_diff>
--- a/dashboard/public/subject_upload_demo.xlsx
+++ b/dashboard/public/subject_upload_demo.xlsx
@@ -8,14 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mutiur\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F66FF902-D901-45E2-A9B9-F6BC7465790E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0B60223-75BD-46D7-91B5-52D86D23DF94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Subjects" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -592,6 +603,7 @@
         <v>33</v>
       </c>
       <c r="E2">
+        <f ca="1">YEAR(TODAY())</f>
         <v>2026</v>
       </c>
       <c r="F2" t="s">
@@ -618,6 +630,7 @@
         <v>17</v>
       </c>
       <c r="E3">
+        <f t="shared" ref="E3:E65" ca="1" si="0">YEAR(TODAY())</f>
         <v>2026</v>
       </c>
       <c r="F3" t="s">
@@ -644,6 +657,7 @@
         <v>33</v>
       </c>
       <c r="E4">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F4" t="s">
@@ -670,6 +684,7 @@
         <v>17</v>
       </c>
       <c r="E5">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F5" t="s">
@@ -696,6 +711,7 @@
         <v>33</v>
       </c>
       <c r="E6">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G6" t="s">
@@ -719,6 +735,7 @@
         <v>33</v>
       </c>
       <c r="E7">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G7" t="s">
@@ -742,6 +759,7 @@
         <v>33</v>
       </c>
       <c r="E8">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G8" t="s">
@@ -765,6 +783,7 @@
         <v>33</v>
       </c>
       <c r="E9">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G9" t="s">
@@ -788,6 +807,7 @@
         <v>17</v>
       </c>
       <c r="E10">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G10" t="s">
@@ -808,6 +828,7 @@
         <v>50</v>
       </c>
       <c r="E11">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G11" t="s">
@@ -831,6 +852,7 @@
         <v>33</v>
       </c>
       <c r="E12">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F12" t="s">
@@ -857,6 +879,7 @@
         <v>17</v>
       </c>
       <c r="E13">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F13" t="s">
@@ -883,6 +906,7 @@
         <v>33</v>
       </c>
       <c r="E14">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F14" t="s">
@@ -909,6 +933,7 @@
         <v>17</v>
       </c>
       <c r="E15">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F15" t="s">
@@ -935,6 +960,7 @@
         <v>33</v>
       </c>
       <c r="E16">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G16" t="s">
@@ -958,6 +984,7 @@
         <v>33</v>
       </c>
       <c r="E17">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G17" t="s">
@@ -981,6 +1008,7 @@
         <v>33</v>
       </c>
       <c r="E18">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G18" t="s">
@@ -1004,6 +1032,7 @@
         <v>33</v>
       </c>
       <c r="E19">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G19" t="s">
@@ -1027,6 +1056,7 @@
         <v>17</v>
       </c>
       <c r="E20">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G20" t="s">
@@ -1047,6 +1077,7 @@
         <v>50</v>
       </c>
       <c r="E21">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G21" t="s">
@@ -1070,6 +1101,7 @@
         <v>33</v>
       </c>
       <c r="E22">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F22" t="s">
@@ -1096,6 +1128,7 @@
         <v>17</v>
       </c>
       <c r="E23">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F23" t="s">
@@ -1122,6 +1155,7 @@
         <v>33</v>
       </c>
       <c r="E24">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F24" t="s">
@@ -1148,6 +1182,7 @@
         <v>17</v>
       </c>
       <c r="E25">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F25" t="s">
@@ -1174,6 +1209,7 @@
         <v>33</v>
       </c>
       <c r="E26">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G26" t="s">
@@ -1197,6 +1233,7 @@
         <v>33</v>
       </c>
       <c r="E27">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G27" t="s">
@@ -1220,6 +1257,7 @@
         <v>33</v>
       </c>
       <c r="E28">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G28" t="s">
@@ -1243,6 +1281,7 @@
         <v>33</v>
       </c>
       <c r="E29">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G29" t="s">
@@ -1266,6 +1305,7 @@
         <v>17</v>
       </c>
       <c r="E30">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G30" t="s">
@@ -1286,6 +1326,7 @@
         <v>50</v>
       </c>
       <c r="E31">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G31" t="s">
@@ -1309,6 +1350,7 @@
         <v>33</v>
       </c>
       <c r="E32">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F32" t="s">
@@ -1347,6 +1389,7 @@
         <v>33</v>
       </c>
       <c r="E33">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F33" t="s">
@@ -1385,6 +1428,7 @@
         <v>33</v>
       </c>
       <c r="E34">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F34" t="s">
@@ -1423,6 +1467,7 @@
         <v>33</v>
       </c>
       <c r="E35">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F35" t="s">
@@ -1461,6 +1506,7 @@
         <v>33</v>
       </c>
       <c r="E36">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G36" t="s">
@@ -1496,6 +1542,7 @@
         <v>33</v>
       </c>
       <c r="E37">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G37" t="s">
@@ -1531,6 +1578,7 @@
         <v>33</v>
       </c>
       <c r="E38">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G38" t="s">
@@ -1569,6 +1617,7 @@
         <v>33</v>
       </c>
       <c r="E39">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G39" t="s">
@@ -1607,6 +1656,7 @@
         <v>33</v>
       </c>
       <c r="E40">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G40" t="s">
@@ -1651,6 +1701,7 @@
         <v>33</v>
       </c>
       <c r="E41">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G41" t="s">
@@ -1689,6 +1740,7 @@
         <v>33</v>
       </c>
       <c r="E42">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G42" t="s">
@@ -1733,6 +1785,7 @@
         <v>33</v>
       </c>
       <c r="E43">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G43" t="s">
@@ -1771,6 +1824,7 @@
         <v>33</v>
       </c>
       <c r="E44">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G44" t="s">
@@ -1815,6 +1869,7 @@
         <v>33</v>
       </c>
       <c r="E45">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G45" t="s">
@@ -1853,6 +1908,7 @@
         <v>8</v>
       </c>
       <c r="E46">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G46" t="s">
@@ -1882,6 +1938,7 @@
         <v>33</v>
       </c>
       <c r="E47">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G47" t="s">
@@ -1926,6 +1983,7 @@
         <v>33</v>
       </c>
       <c r="E48">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G48" t="s">
@@ -1970,6 +2028,7 @@
         <v>33</v>
       </c>
       <c r="E49">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F49" t="s">
@@ -2008,6 +2067,7 @@
         <v>33</v>
       </c>
       <c r="E50">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F50" t="s">
@@ -2046,6 +2106,7 @@
         <v>33</v>
       </c>
       <c r="E51">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F51" t="s">
@@ -2084,6 +2145,7 @@
         <v>33</v>
       </c>
       <c r="E52">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="F52" t="s">
@@ -2122,6 +2184,7 @@
         <v>33</v>
       </c>
       <c r="E53">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G53" t="s">
@@ -2157,6 +2220,7 @@
         <v>33</v>
       </c>
       <c r="E54">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G54" t="s">
@@ -2192,6 +2256,7 @@
         <v>33</v>
       </c>
       <c r="E55">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G55" t="s">
@@ -2230,6 +2295,7 @@
         <v>33</v>
       </c>
       <c r="E56">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G56" t="s">
@@ -2268,6 +2334,7 @@
         <v>33</v>
       </c>
       <c r="E57">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G57" t="s">
@@ -2312,6 +2379,7 @@
         <v>33</v>
       </c>
       <c r="E58">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G58" t="s">
@@ -2350,6 +2418,7 @@
         <v>33</v>
       </c>
       <c r="E59">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G59" t="s">
@@ -2394,6 +2463,7 @@
         <v>33</v>
       </c>
       <c r="E60">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G60" t="s">
@@ -2432,6 +2502,7 @@
         <v>33</v>
       </c>
       <c r="E61">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G61" t="s">
@@ -2476,6 +2547,7 @@
         <v>33</v>
       </c>
       <c r="E62">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G62" t="s">
@@ -2514,6 +2586,7 @@
         <v>8</v>
       </c>
       <c r="E63">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G63" t="s">
@@ -2543,6 +2616,7 @@
         <v>33</v>
       </c>
       <c r="E64">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G64" t="s">
@@ -2587,6 +2661,7 @@
         <v>33</v>
       </c>
       <c r="E65">
+        <f t="shared" ca="1" si="0"/>
         <v>2026</v>
       </c>
       <c r="G65" t="s">
@@ -2620,7 +2695,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D1 A2 C2:D2 E2:F2 G3 H1 E4 G1 E1:F1 E3:F3" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D1 A2 C2:D2 F2 G3 H1 G1 E1:F1 F3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>